<commit_message>
Fix Mark as Unread header styling - blue fill on all merged cells
</commit_message>
<xml_diff>
--- a/Message_List/Message_List_Test_Cases.xlsx
+++ b/Message_List/Message_List_Test_Cases.xlsx
@@ -4925,13 +4925,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B117" s="12" t="n"/>
-      <c r="C117" s="12" t="n"/>
-      <c r="D117" s="12" t="n"/>
-      <c r="E117" s="12" t="n"/>
-      <c r="F117" s="12" t="n"/>
-      <c r="G117" s="12" t="n"/>
-      <c r="H117" s="12" t="n"/>
+      <c r="B117" s="11" t="n"/>
+      <c r="C117" s="11" t="n"/>
+      <c r="D117" s="11" t="n"/>
+      <c r="E117" s="11" t="n"/>
+      <c r="F117" s="11" t="n"/>
+      <c r="G117" s="11" t="n"/>
+      <c r="H117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="9" t="inlineStr">
@@ -6511,13 +6511,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="12" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -7333,13 +7333,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="12" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -7931,13 +7931,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="12" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -8698,13 +8698,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="12" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -9502,13 +9502,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="12" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -10312,13 +10312,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
-      <c r="G17" s="12" t="n"/>
-      <c r="H17" s="12" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Cache bust - force CDN refresh
</commit_message>
<xml_diff>
--- a/Message_List/Message_List_Test_Cases.xlsx
+++ b/Message_List/Message_List_Test_Cases.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +158,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4795,13 +4797,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B114" s="11" t="n"/>
-      <c r="C114" s="11" t="n"/>
-      <c r="D114" s="11" t="n"/>
-      <c r="E114" s="11" t="n"/>
-      <c r="F114" s="11" t="n"/>
-      <c r="G114" s="11" t="n"/>
-      <c r="H114" s="11" t="n"/>
+      <c r="B114" s="13" t="n"/>
+      <c r="C114" s="13" t="n"/>
+      <c r="D114" s="13" t="n"/>
+      <c r="E114" s="13" t="n"/>
+      <c r="F114" s="13" t="n"/>
+      <c r="G114" s="13" t="n"/>
+      <c r="H114" s="14" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
@@ -6551,13 +6553,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="11" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="14" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -7413,13 +7415,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="14" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -8051,13 +8053,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="14" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -8858,13 +8860,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
-      <c r="H18" s="11" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -9702,13 +9704,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="14" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -10552,13 +10554,13 @@
           <t>Mark as Unread</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="11" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="14" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">

</xml_diff>